<commit_message>
Data room: names agree everywhere, team and market read strong, green flags in the answer key with checks
</commit_message>
<xml_diff>
--- a/data_room/hollis_voice/02_financials/financial_model.xlsx
+++ b/data_room/hollis_voice/02_financials/financial_model.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Hiring_Plan" sheetId="6" r:id="rId6"/>
     <sheet name="Cash_Runway" sheetId="7" r:id="rId7"/>
     <sheet name="Cash_Bridge" sheetId="8" r:id="rId8"/>
+    <sheet name="Market" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="ARR_TOTAL">ARR_Build!$E$15</definedName>
@@ -29,6 +30,9 @@
     <definedName name="HOSTING_USD_MONTH">Assumptions!$B$13</definedName>
     <definedName name="LICENCES_PCT">Assumptions!$B$12</definedName>
     <definedName name="LOAD_FACTOR">Assumptions!$B$8</definedName>
+    <definedName name="MARKET_ACV_USD">Market!$B$6</definedName>
+    <definedName name="MARKET_CLINICS">Market!$B$5</definedName>
+    <definedName name="MARKET_TAM_USD">Market!$B$7</definedName>
     <definedName name="NET_LOSS_BEFORE_2025_USD">Assumptions!$B$21</definedName>
     <definedName name="NRR_12M">Cohorts!$E$14</definedName>
     <definedName name="PAYROLL_NOW_USD_MONTH">Assumptions!$B$22</definedName>
@@ -49,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="278">
   <si>
     <t>Hollis Voice: financial model</t>
   </si>
@@ -81,6 +85,9 @@
     <t>Cash_Bridge: money raised, less losses since the company began, equals cash at the data date.</t>
   </si>
   <si>
+    <t>Market: the company's own market estimate, the one the deck's market slide uses.</t>
+  </si>
+  <si>
     <t>Definitions</t>
   </si>
   <si>
@@ -621,7 +628,7 @@
     <t>Implementation Specialist</t>
   </si>
   <si>
-    <t>Head of Sales</t>
+    <t>Director of Enterprise Sales</t>
   </si>
   <si>
     <t>Support Specialist</t>
@@ -633,9 +640,6 @@
     <t>Hires in this plan</t>
   </si>
   <si>
-    <t>Staff after these hires</t>
-  </si>
-  <si>
     <t>Cash and runway (USD)</t>
   </si>
   <si>
@@ -856,6 +860,33 @@
   </si>
   <si>
     <t>Rounding only: the loss before 2025 is stated in whole dollars.</t>
+  </si>
+  <si>
+    <t>Market size (USD)</t>
+  </si>
+  <si>
+    <t>These are the company's own estimates. No outside source is in the room.</t>
+  </si>
+  <si>
+    <t>US independent veterinary clinics (company estimate)</t>
+  </si>
+  <si>
+    <t>The same count as the deck's market slide.</t>
+  </si>
+  <si>
+    <t>Annual contract value per clinic (USD, company estimate)</t>
+  </si>
+  <si>
+    <t>A planning figure for what a clinic pays in a year.</t>
+  </si>
+  <si>
+    <t>Market size: clinics times annual contract value (USD)</t>
+  </si>
+  <si>
+    <t>For comparison: subscription ARR per paying clinic today (USD)</t>
+  </si>
+  <si>
+    <t>Subscription ARR in ARR_Build divided by the paying clinics counted there.</t>
   </si>
 </sst>
 </file>
@@ -1266,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="110.7109375" customWidth="1"/>
@@ -1322,13 +1353,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1">
-      <c r="A13" s="2" t="s">
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:1">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1347,9 +1378,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
-      <c r="A19" s="3" t="s">
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1369,227 +1405,227 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="6">
         <v>1800000</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" s="7">
         <v>0.035</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="6">
         <v>1.28</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" s="6">
         <v>17</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B10" s="6">
         <v>140000</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11" s="7">
         <v>0.15</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="7">
         <v>0.05</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="6">
         <v>20541.29</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" s="6">
         <v>60000</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B15" s="6">
         <v>140000</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B16" s="6">
         <v>9000000</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" s="6">
         <v>4</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" s="6">
         <v>186739</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="6">
         <v>2000000</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B20" s="6">
         <v>3500000</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B21" s="6">
         <v>592499</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22" s="6">
         <f>STAFF_NOW*AVG_BASE_NOW*LOAD_FACTOR/12</f>
         <v>253866.66666666666</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1609,227 +1645,227 @@
   <sheetData>
     <row r="1" spans="1:35">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:35">
       <c r="A4" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="W4" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AA4" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AB4" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AC4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AD4" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AE4" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AF4" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AG4" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AH4" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AI4" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:35">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="R5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="T5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="U5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="V5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W5" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="X5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Y5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Z5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AA5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AB5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AC5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AD5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AE5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AF5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AG5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AH5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AI5" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:35">
       <c r="A6" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -1868,10 +1904,10 @@
     </row>
     <row r="7" spans="1:35">
       <c r="A7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" t="s">
         <v>97</v>
-      </c>
-      <c r="B7" t="s">
-        <v>96</v>
       </c>
       <c r="C7" s="10">
         <v>2651</v>
@@ -1939,10 +1975,10 @@
     </row>
     <row r="8" spans="1:35">
       <c r="A8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
@@ -2010,10 +2046,10 @@
     </row>
     <row r="9" spans="1:35">
       <c r="A9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C9" s="10">
         <v>2500</v>
@@ -2117,10 +2153,10 @@
     </row>
     <row r="10" spans="1:35">
       <c r="A10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C10" s="10">
         <f>C7+C8</f>
@@ -2245,10 +2281,10 @@
     </row>
     <row r="11" spans="1:35">
       <c r="A11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C11" s="10">
         <f>C10+C9</f>
@@ -2385,7 +2421,7 @@
     </row>
     <row r="12" spans="1:35">
       <c r="A12" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -2424,10 +2460,10 @@
     </row>
     <row r="13" spans="1:35">
       <c r="A13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C13" s="10">
         <v>435.7</v>
@@ -2531,10 +2567,10 @@
     </row>
     <row r="14" spans="1:35">
       <c r="A14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" t="s">
         <v>105</v>
-      </c>
-      <c r="B14" t="s">
-        <v>104</v>
       </c>
       <c r="C14" s="10">
         <v>148.48</v>
@@ -2638,10 +2674,10 @@
     </row>
     <row r="15" spans="1:35">
       <c r="A15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" s="10">
         <f>C13+C14</f>
@@ -2778,7 +2814,7 @@
     </row>
     <row r="16" spans="1:35">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C16" s="11">
         <f>C10-C15</f>
@@ -2915,7 +2951,7 @@
     </row>
     <row r="17" spans="1:35">
       <c r="A17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C17" s="12">
         <f>C16/C10</f>
@@ -3052,7 +3088,7 @@
     </row>
     <row r="18" spans="1:35">
       <c r="A18" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -3091,10 +3127,10 @@
     </row>
     <row r="19" spans="1:35">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C19" s="10">
         <v>31186.59</v>
@@ -3198,10 +3234,10 @@
     </row>
     <row r="20" spans="1:35">
       <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" t="s">
         <v>112</v>
-      </c>
-      <c r="B20" t="s">
-        <v>111</v>
       </c>
       <c r="C20" s="10">
         <v>384.59</v>
@@ -3305,10 +3341,10 @@
     </row>
     <row r="21" spans="1:35">
       <c r="A21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C21" s="10">
         <v>14987.33</v>
@@ -3412,10 +3448,10 @@
     </row>
     <row r="22" spans="1:35">
       <c r="A22" t="s">
+        <v>116</v>
+      </c>
+      <c r="B22" t="s">
         <v>115</v>
-      </c>
-      <c r="B22" t="s">
-        <v>114</v>
       </c>
       <c r="C22" s="10">
         <v>0</v>
@@ -3519,10 +3555,10 @@
     </row>
     <row r="23" spans="1:35">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C23" s="10">
         <v>0</v>
@@ -3626,10 +3662,10 @@
     </row>
     <row r="24" spans="1:35">
       <c r="A24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C24" s="10">
         <v>15663.86</v>
@@ -3733,10 +3769,10 @@
     </row>
     <row r="25" spans="1:35">
       <c r="A25" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" t="s">
         <v>119</v>
-      </c>
-      <c r="B25" t="s">
-        <v>118</v>
       </c>
       <c r="C25" s="10">
         <v>29694.61</v>
@@ -3840,7 +3876,7 @@
     </row>
     <row r="26" spans="1:35">
       <c r="A26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C26" s="11">
         <f>C19+C20+C21+C22+C23+C24+C25</f>
@@ -3977,7 +4013,7 @@
     </row>
     <row r="27" spans="1:35">
       <c r="A27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C27" s="11">
         <f>C16+C9-C26</f>
@@ -4114,7 +4150,7 @@
     </row>
     <row r="28" spans="1:35">
       <c r="A28" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -4153,10 +4189,10 @@
     </row>
     <row r="29" spans="1:35">
       <c r="A29" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" t="s">
         <v>123</v>
-      </c>
-      <c r="B29" t="s">
-        <v>122</v>
       </c>
       <c r="C29" s="10">
         <f>C19+C21+C22+C24</f>
@@ -4293,10 +4329,10 @@
     </row>
     <row r="30" spans="1:35">
       <c r="A30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C30" s="10">
         <f>-C27</f>
@@ -4433,10 +4469,10 @@
     </row>
     <row r="31" spans="1:35">
       <c r="A31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B31" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C31" s="10">
         <v>4</v>
@@ -4501,46 +4537,10 @@
       <c r="W31" s="10">
         <v>17</v>
       </c>
-      <c r="X31" s="10">
-        <v>19</v>
-      </c>
-      <c r="Y31" s="10">
-        <v>21</v>
-      </c>
-      <c r="Z31" s="10">
-        <v>23</v>
-      </c>
-      <c r="AA31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AB31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AC31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AD31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AE31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AF31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AG31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AH31" s="10">
-        <v>25</v>
-      </c>
-      <c r="AI31" s="10">
-        <v>25</v>
-      </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -4561,40 +4561,40 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C5" s="10">
         <v>13</v>
@@ -4607,15 +4607,15 @@
         <v>121044</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C6" s="10">
         <v>14</v>
@@ -4628,15 +4628,15 @@
         <v>126420</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C7" s="10">
         <v>21</v>
@@ -4649,15 +4649,15 @@
         <v>167820</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C8" s="10">
         <v>32</v>
@@ -4670,15 +4670,15 @@
         <v>648864</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C9" s="10">
         <v>36</v>
@@ -4691,15 +4691,15 @@
         <v>290532</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C10" s="10">
         <v>40</v>
@@ -4712,15 +4712,15 @@
         <v>321060</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C11" s="10">
         <v>56</v>
@@ -4733,15 +4733,15 @@
         <v>385128</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C12" s="11">
         <f>SUM(C5:C11)</f>
@@ -4758,10 +4758,10 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C13" s="10">
         <v>1</v>
@@ -4774,15 +4774,15 @@
         <v>180000</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C14" s="10">
         <v>19</v>
@@ -4794,12 +4794,12 @@
         <v>0</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E15" s="6">
         <f>E12+E13+E14</f>
@@ -4808,27 +4808,27 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C19" s="10">
         <v>2651</v>
@@ -4843,7 +4843,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C20" s="10">
         <v>6828</v>
@@ -4858,7 +4858,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C21" s="10">
         <v>10024</v>
@@ -4873,7 +4873,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C22" s="10">
         <v>12366</v>
@@ -4888,7 +4888,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C23" s="10">
         <v>16059</v>
@@ -4903,7 +4903,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C24" s="10">
         <v>19462</v>
@@ -4918,7 +4918,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C25" s="10">
         <v>23092</v>
@@ -4933,7 +4933,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C26" s="10">
         <v>28610</v>
@@ -4948,7 +4948,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C27" s="10">
         <v>34539</v>
@@ -4963,7 +4963,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C28" s="10">
         <v>40585</v>
@@ -4978,7 +4978,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C29" s="10">
         <v>65867</v>
@@ -4993,7 +4993,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C30" s="10">
         <v>72656</v>
@@ -5008,7 +5008,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C31" s="10">
         <v>77134</v>
@@ -5023,7 +5023,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C32" s="10">
         <v>85778</v>
@@ -5038,7 +5038,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C33" s="10">
         <v>95824</v>
@@ -5053,7 +5053,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C34" s="10">
         <v>122664</v>
@@ -5068,7 +5068,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C35" s="10">
         <v>133652</v>
@@ -5083,7 +5083,7 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C36" s="10">
         <v>142497</v>
@@ -5098,7 +5098,7 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C37" s="10">
         <v>149831</v>
@@ -5113,7 +5113,7 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C38" s="10">
         <v>160971</v>
@@ -5128,7 +5128,7 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C39" s="10">
         <v>171739</v>
@@ -5143,7 +5143,7 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -5163,73 +5163,73 @@
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:18">
       <c r="A4" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:18">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="10">
         <v>4</v>
@@ -5286,7 +5286,7 @@
     </row>
     <row r="6" spans="1:18">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B6" s="10">
         <v>6</v>
@@ -5343,7 +5343,7 @@
     </row>
     <row r="7" spans="1:18">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="10">
         <v>4</v>
@@ -5400,7 +5400,7 @@
     </row>
     <row r="8" spans="1:18">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="10">
         <v>7</v>
@@ -5457,7 +5457,7 @@
     </row>
     <row r="9" spans="1:18">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B9" s="10">
         <v>5</v>
@@ -5514,7 +5514,7 @@
     </row>
     <row r="10" spans="1:18">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B10" s="10">
         <v>6</v>
@@ -5571,7 +5571,7 @@
     </row>
     <row r="11" spans="1:18">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" s="10">
         <v>8</v>
@@ -5628,7 +5628,7 @@
     </row>
     <row r="12" spans="1:18">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B12" s="10">
         <v>8</v>
@@ -5685,7 +5685,7 @@
     </row>
     <row r="13" spans="1:18">
       <c r="A13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B13" s="10">
         <v>9</v>
@@ -5742,7 +5742,7 @@
     </row>
     <row r="14" spans="1:18">
       <c r="A14" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B14" s="11">
         <f>SUM(B5:B13)</f>
@@ -5763,7 +5763,7 @@
     </row>
     <row r="16" spans="1:18">
       <c r="A16" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -5783,40 +5783,40 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D5" s="10">
         <v>191000</v>
@@ -5828,13 +5828,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D6" s="10">
         <v>139000</v>
@@ -5846,13 +5846,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D7" s="10">
         <v>189000</v>
@@ -5864,13 +5864,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D8" s="10">
         <v>141000</v>
@@ -5882,13 +5882,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D9" s="10">
         <v>173500</v>
@@ -5900,13 +5900,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D10" s="10">
         <v>156500</v>
@@ -5918,13 +5918,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D11" s="10">
         <v>211000</v>
@@ -5936,13 +5936,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B12" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D12" s="10">
         <v>119000</v>
@@ -5954,25 +5954,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B13" s="6">
         <f>COUNTA(A5:A12)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="B14" s="10">
-        <f>STAFF_NOW+B13</f>
-        <v>25</v>
-      </c>
-    </row>
     <row r="16" spans="1:5">
       <c r="A16" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -6014,7 +6005,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="6">
         <f>CASH_START</f>
@@ -6023,7 +6014,7 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>198</v>
@@ -6032,16 +6023,16 @@
         <v>199</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>200</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>201</v>
@@ -6055,7 +6046,7 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B8" s="10">
         <v>0</v>
@@ -6067,7 +6058,7 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B9" s="10">
         <v>1</v>
@@ -6101,7 +6092,7 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B10" s="10">
         <v>2</v>
@@ -6135,7 +6126,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B11" s="10">
         <v>3</v>
@@ -6169,7 +6160,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B12" s="10">
         <v>4</v>
@@ -6203,7 +6194,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B13" s="10">
         <v>5</v>
@@ -6237,7 +6228,7 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B14" s="10">
         <v>6</v>
@@ -6271,7 +6262,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="10">
         <v>7</v>
@@ -6305,7 +6296,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B16" s="10">
         <v>8</v>
@@ -6339,7 +6330,7 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B17" s="10">
         <v>9</v>
@@ -6373,7 +6364,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B18" s="10">
         <v>10</v>
@@ -6407,7 +6398,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B19" s="10">
         <v>11</v>
@@ -6441,7 +6432,7 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B20" s="10">
         <v>12</v>
@@ -8107,7 +8098,7 @@
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -8137,13 +8128,13 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>254</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -8238,7 +8229,91 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="60.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="90.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>271</v>
+      </c>
+      <c r="B5" s="6">
+        <v>28000</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>273</v>
+      </c>
+      <c r="B6" s="6">
+        <v>9000</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B7" s="6">
+        <f>MARKET_CLINICS*MARKET_ACV_USD</f>
+        <v>252000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>276</v>
+      </c>
+      <c r="B8" s="10">
+        <f>ARR_Build!E12/ARR_Build!C12</f>
+        <v>9721.075471698114</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>